<commit_message>
Fix: Dialogues and Objective Banner to better help with story flow
</commit_message>
<xml_diff>
--- a/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
+++ b/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR\Unity Projects\Class Assignments\CS 425\CS425-Senior-Project\Assets\Dialogue\Import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337C6272-0D6B-4589-9054-5720CA806C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB519FDC-1C7C-4C58-B237-4AF334E4028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6060" yWindow="1608" windowWidth="18432" windowHeight="12540" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="1440" windowWidth="18432" windowHeight="12540" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="180">
   <si>
     <t>Bound Spirit Dialogue Workbook</t>
   </si>
@@ -446,9 +446,6 @@
     <t>If you happen to find something like that nearby… could you bring it to me?</t>
   </si>
   <si>
-    <t>It was soft… delicate… and carried a sweet scent.</t>
-  </si>
-  <si>
     <t>Ghost1Wrong.asset</t>
   </si>
   <si>
@@ -500,9 +497,6 @@
     <t>What happened to me? How did I die?</t>
   </si>
   <si>
-    <t>The stone beneath the gate is worn smooth by time.</t>
-  </si>
-  <si>
     <t>Three faint markings are carved into its surface.</t>
   </si>
   <si>
@@ -512,9 +506,6 @@
     <t>“Three memories linger in this graveyard. Return what was lost… and the path will open.”</t>
   </si>
   <si>
-    <t>The carving beneath the gate is still visible.</t>
-  </si>
-  <si>
     <t>“Three memories… Return what was lost, and the path will open.”</t>
   </si>
   <si>
@@ -533,28 +524,43 @@
     <t>I'm missing something.</t>
   </si>
   <si>
-    <t>Akila... that's my name. I need to find out more.</t>
-  </si>
-  <si>
-    <t>I need to find out more.</t>
-  </si>
-  <si>
     <t>Wait... this tombstone... Let me read it closer.</t>
   </si>
   <si>
     <t>Every year... when the weather grew warm... I used to bring something here.</t>
   </si>
   <si>
-    <t>… You can see me?</t>
-  </si>
-  <si>
     <t>Chapter0_blockedBeforeGateClue</t>
   </si>
   <si>
-    <t>There is something by the gate that I need to see first.</t>
-  </si>
-  <si>
     <t>BlockedBeforeGateClue.asset</t>
+  </si>
+  <si>
+    <t>The carving is still visible.</t>
+  </si>
+  <si>
+    <t>There is a worn stone around the gate. I should go look at it to help me open this.</t>
+  </si>
+  <si>
+    <t>Looks like I should talk to these three memories before leaving this graveyard.</t>
+  </si>
+  <si>
+    <t>...You can see me?</t>
+  </si>
+  <si>
+    <t>It was soft… delicate… and carried a floral scent.</t>
+  </si>
+  <si>
+    <t>Did you find what once carried that floral scent?</t>
+  </si>
+  <si>
+    <t>This stone besides the gate is worn smooth by time.</t>
+  </si>
+  <si>
+    <t>Akila... that's my name. I need to get out of this graveyard.</t>
+  </si>
+  <si>
+    <t>I need to find out more. I need to leave this graveyard.</t>
   </si>
 </sst>
 </file>
@@ -1069,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -1181,7 +1187,7 @@
         <v>57</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -1202,22 +1208,20 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D6" s="6">
         <v>0</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="E6" s="6"/>
       <c r="F6" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1237,11 +1241,9 @@
       <c r="D7" s="6">
         <v>0</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="E7" s="6"/>
       <c r="F7" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -1261,11 +1263,9 @@
       <c r="D8" s="6">
         <v>1</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="E8" s="6"/>
       <c r="F8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -1285,11 +1285,9 @@
       <c r="D9" s="6">
         <v>2</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="E9" s="6"/>
       <c r="F9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
@@ -1309,11 +1307,9 @@
       <c r="D10" s="6">
         <v>3</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="E10" s="6"/>
       <c r="F10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -1322,22 +1318,22 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="D11" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
@@ -1355,13 +1351,13 @@
         <v>72</v>
       </c>
       <c r="D12" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -1369,36 +1365,36 @@
       <c r="J12" s="6"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
+      <c r="A13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>161</v>
+      </c>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="6">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>92</v>
-      </c>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
@@ -1415,13 +1411,13 @@
         <v>61</v>
       </c>
       <c r="D15" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
@@ -1439,13 +1435,13 @@
         <v>61</v>
       </c>
       <c r="D16" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
@@ -1463,13 +1459,13 @@
         <v>61</v>
       </c>
       <c r="D17" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
@@ -1487,13 +1483,13 @@
         <v>61</v>
       </c>
       <c r="D18" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>158</v>
+        <v>64</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
@@ -1511,13 +1507,13 @@
         <v>61</v>
       </c>
       <c r="D19" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>65</v>
+        <v>157</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -1535,13 +1531,13 @@
         <v>61</v>
       </c>
       <c r="D20" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>171</v>
+        <v>65</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
@@ -1550,22 +1546,22 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="D21" s="6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F21" t="s">
-        <v>170</v>
+      <c r="F21" s="6" t="s">
+        <v>179</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
@@ -1573,36 +1569,36 @@
       <c r="J21" s="6"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
+      <c r="A22" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="6">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" t="s">
+        <v>178</v>
+      </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D23" s="6">
-        <v>0</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>174</v>
-      </c>
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6"/>
@@ -1619,13 +1615,13 @@
         <v>42</v>
       </c>
       <c r="D24" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>43</v>
+        <v>174</v>
       </c>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
@@ -1643,13 +1639,13 @@
         <v>42</v>
       </c>
       <c r="D25" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F25" t="s">
-        <v>173</v>
+        <v>148</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
@@ -1667,13 +1663,13 @@
         <v>42</v>
       </c>
       <c r="D26" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F26" t="s">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
@@ -1691,13 +1687,13 @@
         <v>42</v>
       </c>
       <c r="D27" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F27" t="s">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
@@ -1706,22 +1702,22 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
-        <v>150</v>
+        <v>41</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>151</v>
+        <v>42</v>
       </c>
       <c r="D28" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>157</v>
+        <v>148</v>
+      </c>
+      <c r="F28" t="s">
+        <v>140</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
@@ -1730,22 +1726,22 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>44</v>
+        <v>149</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>45</v>
+        <v>150</v>
       </c>
       <c r="D29" s="6">
         <v>0</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>46</v>
+        <v>176</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -1763,13 +1759,13 @@
         <v>45</v>
       </c>
       <c r="D30" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
@@ -1787,13 +1783,13 @@
         <v>45</v>
       </c>
       <c r="D31" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
@@ -1802,22 +1798,22 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D32" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
@@ -1835,13 +1831,13 @@
         <v>50</v>
       </c>
       <c r="D33" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>148</v>
+        <v>51</v>
       </c>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
@@ -1859,13 +1855,13 @@
         <v>50</v>
       </c>
       <c r="D34" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>52</v>
+        <v>147</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
@@ -1883,13 +1879,13 @@
         <v>50</v>
       </c>
       <c r="D35" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>147</v>
+        <v>52</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
@@ -1907,13 +1903,13 @@
         <v>50</v>
       </c>
       <c r="D36" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>53</v>
+        <v>146</v>
       </c>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
@@ -1922,22 +1918,22 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
-        <v>142</v>
+        <v>49</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>143</v>
+        <v>50</v>
       </c>
       <c r="D37" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F37" t="s">
-        <v>144</v>
+        <v>148</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>53</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
@@ -1946,75 +1942,75 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="6" t="s">
+      <c r="D38" s="6">
+        <v>0</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="F38" t="s">
         <v>143</v>
       </c>
-      <c r="D38" s="6">
-        <v>1</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F38" t="s">
-        <v>145</v>
-      </c>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>143</v>
-      </c>
       <c r="D39" s="6">
+        <v>1</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="F39" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D40" s="6">
         <v>2</v>
       </c>
-      <c r="E39" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="F39" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" s="6"/>
-      <c r="B40" s="6"/>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
-      <c r="J40" s="6"/>
+      <c r="E40" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="F40" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D41" s="6">
-        <v>0</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F41" t="s">
-        <v>106</v>
-      </c>
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
       <c r="I41" s="6"/>
@@ -2031,13 +2027,13 @@
         <v>97</v>
       </c>
       <c r="D42" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F42" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
@@ -2055,13 +2051,13 @@
         <v>97</v>
       </c>
       <c r="D43" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
@@ -2079,13 +2075,13 @@
         <v>97</v>
       </c>
       <c r="D44" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F44" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
@@ -2103,13 +2099,13 @@
         <v>97</v>
       </c>
       <c r="D45" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F45" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
@@ -2118,22 +2114,22 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>152</v>
+        <v>94</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>153</v>
+        <v>97</v>
       </c>
       <c r="D46" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F46" t="s">
-        <v>154</v>
+        <v>109</v>
       </c>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
@@ -2142,13 +2138,13 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
-        <v>95</v>
+        <v>151</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>98</v>
+        <v>152</v>
       </c>
       <c r="D47" s="6">
         <v>0</v>
@@ -2157,7 +2153,7 @@
         <v>100</v>
       </c>
       <c r="F47" t="s">
-        <v>101</v>
+        <v>153</v>
       </c>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
@@ -2175,13 +2171,13 @@
         <v>98</v>
       </c>
       <c r="D48" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F48" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
@@ -2199,13 +2195,13 @@
         <v>98</v>
       </c>
       <c r="D49" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F49" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
@@ -2214,22 +2210,22 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D50" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F50" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
@@ -2247,13 +2243,13 @@
         <v>99</v>
       </c>
       <c r="D51" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F51" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
@@ -2271,13 +2267,13 @@
         <v>99</v>
       </c>
       <c r="D52" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F52" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
@@ -2295,13 +2291,13 @@
         <v>99</v>
       </c>
       <c r="D53" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F53" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -2310,22 +2306,22 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D54" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F54" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
@@ -2343,14 +2339,18 @@
         <v>104</v>
       </c>
       <c r="D55" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F55" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
@@ -2363,38 +2363,34 @@
         <v>104</v>
       </c>
       <c r="D56" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F56" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D57" s="6">
+        <v>2</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F57" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A58" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="D58" s="6">
-        <v>0</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="F58" t="s">
-        <v>119</v>
-      </c>
-      <c r="G58" s="6"/>
-      <c r="H58" s="6"/>
-      <c r="I58" s="6"/>
-      <c r="J58" s="6"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
@@ -2407,13 +2403,13 @@
         <v>135</v>
       </c>
       <c r="D59" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F59" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
@@ -2431,13 +2427,13 @@
         <v>135</v>
       </c>
       <c r="D60" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F60" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
@@ -2455,13 +2451,13 @@
         <v>135</v>
       </c>
       <c r="D61" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F61" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
@@ -2479,13 +2475,13 @@
         <v>135</v>
       </c>
       <c r="D62" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F62" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
@@ -2494,22 +2490,22 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
-        <v>155</v>
+        <v>105</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="D63" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F63" t="s">
-        <v>157</v>
+        <v>124</v>
       </c>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
@@ -2518,13 +2514,13 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="D64" s="6">
         <v>0</v>
@@ -2533,7 +2529,7 @@
         <v>120</v>
       </c>
       <c r="F64" t="s">
-        <v>130</v>
+        <v>156</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
@@ -2551,13 +2547,13 @@
         <v>136</v>
       </c>
       <c r="D65" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F65" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G65" s="6"/>
       <c r="H65" s="6"/>
@@ -2566,22 +2562,22 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D66" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F66" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G66" s="6"/>
       <c r="H66" s="6"/>
@@ -2599,13 +2595,13 @@
         <v>137</v>
       </c>
       <c r="D67" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F67" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G67" s="6"/>
       <c r="H67" s="6"/>
@@ -2623,13 +2619,13 @@
         <v>137</v>
       </c>
       <c r="D68" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F68" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G68" s="6"/>
       <c r="H68" s="6"/>
@@ -2647,13 +2643,13 @@
         <v>137</v>
       </c>
       <c r="D69" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F69" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G69" s="6"/>
       <c r="H69" s="6"/>
@@ -2662,22 +2658,22 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D70" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F70" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="G70" s="6"/>
       <c r="H70" s="6"/>
@@ -2695,45 +2691,45 @@
         <v>138</v>
       </c>
       <c r="D71" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F71" t="s">
+        <v>125</v>
+      </c>
+      <c r="G71" s="6"/>
+      <c r="H71" s="6"/>
+      <c r="I71" s="6"/>
+      <c r="J71" s="6"/>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A72" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D72" s="6">
+        <v>1</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F72" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A72" s="6"/>
-      <c r="B72" s="6"/>
-      <c r="C72" s="6"/>
-      <c r="D72" s="6"/>
-      <c r="E72" s="6"/>
-    </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A73" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B73" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C73" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D73" s="6">
-        <v>0</v>
-      </c>
-      <c r="E73" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F73" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="G73" s="6"/>
-      <c r="H73" s="6"/>
-      <c r="I73" s="6"/>
-      <c r="J73" s="6"/>
+      <c r="A73" s="6"/>
+      <c r="B73" s="6"/>
+      <c r="C73" s="6"/>
+      <c r="D73" s="6"/>
+      <c r="E73" s="6"/>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
@@ -2746,13 +2742,13 @@
         <v>67</v>
       </c>
       <c r="D74" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
@@ -2770,13 +2766,13 @@
         <v>67</v>
       </c>
       <c r="D75" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
@@ -2785,22 +2781,22 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B76" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D76" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>70</v>
+        <v>166</v>
       </c>
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
@@ -2808,36 +2804,36 @@
       <c r="J76" s="6"/>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A77" s="6"/>
-      <c r="B77" s="6"/>
-      <c r="C77" s="6"/>
-      <c r="D77" s="6"/>
-      <c r="E77" s="6"/>
-      <c r="F77" s="6"/>
+      <c r="A77" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D77" s="6">
+        <v>0</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>70</v>
+      </c>
       <c r="G77" s="6"/>
       <c r="H77" s="6"/>
       <c r="I77" s="6"/>
       <c r="J77" s="6"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A78" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B78" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D78" s="6">
-        <v>0</v>
-      </c>
-      <c r="E78" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F78" s="6" t="s">
-        <v>75</v>
-      </c>
+      <c r="A78" s="6"/>
+      <c r="B78" s="6"/>
+      <c r="C78" s="6"/>
+      <c r="D78" s="6"/>
+      <c r="E78" s="6"/>
+      <c r="F78" s="6"/>
       <c r="G78" s="6"/>
       <c r="H78" s="6"/>
       <c r="I78" s="6"/>
@@ -2845,13 +2841,13 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D79" s="6">
         <v>0</v>
@@ -2860,7 +2856,7 @@
         <v>40</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>165</v>
+        <v>75</v>
       </c>
       <c r="G79" s="6"/>
       <c r="H79" s="6"/>
@@ -2869,22 +2865,22 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D80" s="6">
         <v>0</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="G80" s="6"/>
       <c r="H80" s="6"/>
@@ -2893,22 +2889,22 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D81" s="6">
         <v>0</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>84</v>
+        <v>163</v>
       </c>
       <c r="G81" s="6"/>
       <c r="H81" s="6"/>
@@ -2916,36 +2912,40 @@
       <c r="J81" s="6"/>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A82" s="6"/>
-      <c r="B82" s="6"/>
-      <c r="C82" s="6"/>
-      <c r="D82" s="6"/>
-      <c r="E82" s="6"/>
-      <c r="F82" s="6"/>
+      <c r="A82" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D82" s="6">
+        <v>0</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>84</v>
+      </c>
       <c r="G82" s="6"/>
       <c r="H82" s="6"/>
       <c r="I82" s="6"/>
       <c r="J82" s="6"/>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>85</v>
-      </c>
-      <c r="B83" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C83" t="s">
-        <v>86</v>
-      </c>
-      <c r="D83">
-        <v>0</v>
-      </c>
-      <c r="E83" t="s">
-        <v>40</v>
-      </c>
-      <c r="F83" t="s">
-        <v>88</v>
-      </c>
+      <c r="A83" s="6"/>
+      <c r="B83" s="6"/>
+      <c r="C83" s="6"/>
+      <c r="D83" s="6"/>
+      <c r="E83" s="6"/>
+      <c r="F83" s="6"/>
+      <c r="G83" s="6"/>
+      <c r="H83" s="6"/>
+      <c r="I83" s="6"/>
+      <c r="J83" s="6"/>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
@@ -2958,13 +2958,13 @@
         <v>86</v>
       </c>
       <c r="D84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E84" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="F84" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
@@ -2978,13 +2978,13 @@
         <v>86</v>
       </c>
       <c r="D85">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E85" t="s">
         <v>87</v>
       </c>
       <c r="F85" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
@@ -2998,21 +2998,34 @@
         <v>86</v>
       </c>
       <c r="D86">
+        <v>2</v>
+      </c>
+      <c r="E86" t="s">
+        <v>87</v>
+      </c>
+      <c r="F86" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>85</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C87" t="s">
+        <v>86</v>
+      </c>
+      <c r="D87">
         <v>3</v>
       </c>
-      <c r="E86" t="s">
+      <c r="E87" t="s">
         <v>40</v>
       </c>
-      <c r="F86" t="s">
+      <c r="F87" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A92" s="6"/>
-      <c r="B92" s="6"/>
-      <c r="C92" s="6"/>
-      <c r="D92" s="6"/>
-      <c r="E92" s="6"/>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="6"/>
@@ -3021,6 +3034,13 @@
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
     </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A94" s="6"/>
+      <c r="B94" s="6"/>
+      <c r="C94" s="6"/>
+      <c r="D94" s="6"/>
+      <c r="E94" s="6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add: Player can see a preview of the gatepuzzle but not to solve them before finished with the ghost offering
</commit_message>
<xml_diff>
--- a/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
+++ b/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR\Unity Projects\Class Assignments\CS 425\CS425-Senior-Project\Assets\Dialogue\Import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB519FDC-1C7C-4C58-B237-4AF334E4028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073F155D-D842-47E5-8F62-D10E89505082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="1440" windowWidth="18432" windowHeight="12540" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="180">
   <si>
     <t>Bound Spirit Dialogue Workbook</t>
   </si>
@@ -509,9 +509,6 @@
     <t>“Three memories… Return what was lost, and the path will open.”</t>
   </si>
   <si>
-    <t>There's some sort of seal on the gate. Maybe there's a clue nearby...</t>
-  </si>
-  <si>
     <t>Leaving already? I don't even remember who I am…</t>
   </si>
   <si>
@@ -539,12 +536,6 @@
     <t>The carving is still visible.</t>
   </si>
   <si>
-    <t>There is a worn stone around the gate. I should go look at it to help me open this.</t>
-  </si>
-  <si>
-    <t>Looks like I should talk to these three memories before leaving this graveyard.</t>
-  </si>
-  <si>
     <t>...You can see me?</t>
   </si>
   <si>
@@ -561,6 +552,15 @@
   </si>
   <si>
     <t>I need to find out more. I need to leave this graveyard.</t>
+  </si>
+  <si>
+    <t>Now that I have helped the three spirits, I should know how to solve this.</t>
+  </si>
+  <si>
+    <t>There is a worn stone around the gate. I should go look at it to help me solve this.</t>
+  </si>
+  <si>
+    <t>Looks like I should talk to these three memories before being able too leave this graveyard.</t>
   </si>
 </sst>
 </file>
@@ -1187,7 +1187,7 @@
         <v>57</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -1208,20 +1208,22 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D6" s="6">
         <v>0</v>
       </c>
-      <c r="E6" s="6"/>
+      <c r="E6" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="F6" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1243,7 +1245,7 @@
       </c>
       <c r="E7" s="6"/>
       <c r="F7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -1333,7 +1335,7 @@
         <v>40</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
@@ -1357,7 +1359,7 @@
         <v>40</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -1561,7 +1563,7 @@
         <v>40</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
@@ -1585,7 +1587,7 @@
         <v>40</v>
       </c>
       <c r="F22" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
@@ -1621,7 +1623,7 @@
         <v>148</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
@@ -1669,7 +1671,7 @@
         <v>148</v>
       </c>
       <c r="F26" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
@@ -1693,7 +1695,7 @@
         <v>148</v>
       </c>
       <c r="F27" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
@@ -1741,7 +1743,7 @@
         <v>148</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -2748,7 +2750,7 @@
         <v>40</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
@@ -2772,7 +2774,7 @@
         <v>40</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
@@ -2796,7 +2798,7 @@
         <v>40</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
@@ -2880,7 +2882,7 @@
         <v>40</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="G80" s="6"/>
       <c r="H80" s="6"/>
@@ -2904,7 +2906,7 @@
         <v>57</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G81" s="6"/>
       <c r="H81" s="6"/>

</xml_diff>

<commit_message>
Fix: Change shiny color and scale it up. Shiny also persist throughout the scene, independent of the player location
</commit_message>
<xml_diff>
--- a/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
+++ b/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR\Unity Projects\Class Assignments\CS 425\CS425-Senior-Project\Assets\Dialogue\Import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073F155D-D842-47E5-8F62-D10E89505082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F17AAC3-F3D3-40A4-B24B-A779522BE6C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="1440" windowWidth="18432" windowHeight="12540" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -491,9 +491,6 @@
     <t>Ghost3NeedRepeat</t>
   </si>
   <si>
-    <t>Did you find what once carried that sweet scent?</t>
-  </si>
-  <si>
     <t>What happened to me? How did I die?</t>
   </si>
   <si>
@@ -561,6 +558,9 @@
   </si>
   <si>
     <t>Looks like I should talk to these three memories before being able too leave this graveyard.</t>
+  </si>
+  <si>
+    <t>Did you find the small metal that was once in my hands?</t>
   </si>
 </sst>
 </file>
@@ -1187,7 +1187,7 @@
         <v>57</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -1208,13 +1208,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D6" s="6">
         <v>0</v>
@@ -1223,7 +1223,7 @@
         <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="E7" s="6"/>
       <c r="F7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E8" s="6"/>
       <c r="F8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E9" s="6"/>
       <c r="F9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="E10" s="6"/>
       <c r="F10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -1335,7 +1335,7 @@
         <v>40</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
@@ -1359,7 +1359,7 @@
         <v>40</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -1383,7 +1383,7 @@
         <v>40</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
@@ -1515,7 +1515,7 @@
         <v>40</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -1563,7 +1563,7 @@
         <v>40</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
@@ -1587,7 +1587,7 @@
         <v>40</v>
       </c>
       <c r="F22" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
@@ -1623,7 +1623,7 @@
         <v>148</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
@@ -1671,7 +1671,7 @@
         <v>148</v>
       </c>
       <c r="F26" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
@@ -1695,7 +1695,7 @@
         <v>148</v>
       </c>
       <c r="F27" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
@@ -1743,7 +1743,7 @@
         <v>148</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -2531,7 +2531,7 @@
         <v>120</v>
       </c>
       <c r="F64" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
@@ -2750,7 +2750,7 @@
         <v>40</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
@@ -2774,7 +2774,7 @@
         <v>40</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
@@ -2798,7 +2798,7 @@
         <v>40</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
@@ -2882,7 +2882,7 @@
         <v>40</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G80" s="6"/>
       <c r="H80" s="6"/>
@@ -2906,7 +2906,7 @@
         <v>57</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G81" s="6"/>
       <c r="H81" s="6"/>

</xml_diff>

<commit_message>
Fix: Update Dialogues for ghost before gateHint and Ghost3 offering Hint
</commit_message>
<xml_diff>
--- a/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
+++ b/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR\Unity Projects\Class Assignments\CS 425\CS425-Senior-Project\Assets\Dialogue\Import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073F155D-D842-47E5-8F62-D10E89505082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C02381-D37A-4F00-B6A6-D3F5B44253B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="1440" windowWidth="18432" windowHeight="12540" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="183">
   <si>
     <t>Bound Spirit Dialogue Workbook</t>
   </si>
@@ -401,9 +401,6 @@
     <t>No… that is not what I lost.</t>
   </si>
   <si>
-    <t>What I remember was small… heavy… and cold.</t>
-  </si>
-  <si>
     <t>...Yes. This is the one.</t>
   </si>
   <si>
@@ -491,9 +488,6 @@
     <t>Ghost3NeedRepeat</t>
   </si>
   <si>
-    <t>Did you find what once carried that sweet scent?</t>
-  </si>
-  <si>
     <t>What happened to me? How did I die?</t>
   </si>
   <si>
@@ -557,10 +551,25 @@
     <t>Now that I have helped the three spirits, I should know how to solve this.</t>
   </si>
   <si>
-    <t>There is a worn stone around the gate. I should go look at it to help me solve this.</t>
-  </si>
-  <si>
-    <t>Looks like I should talk to these three memories before being able too leave this graveyard.</t>
+    <t>Did you find the small metal that was once in my hands?</t>
+  </si>
+  <si>
+    <t>There is a worn stone around the gate. I should go look at it, maybe it'll help me…</t>
+  </si>
+  <si>
+    <t>Looks like I need to talk to these three memories before being able too leave this graveyard.</t>
+  </si>
+  <si>
+    <t>What I remember was small... and cold.</t>
+  </si>
+  <si>
+    <t>Chapter0_ghostBlockedBeforeGateClue</t>
+  </si>
+  <si>
+    <t>ghostBlockedBeforeGateClue.asset</t>
+  </si>
+  <si>
+    <t>I don't want to talk to them right now. I just want to get out of here.</t>
   </si>
 </sst>
 </file>
@@ -1075,10 +1084,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="1" max="1" width="31.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="35.21875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
@@ -1187,7 +1196,7 @@
         <v>57</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -1208,13 +1217,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D6" s="6">
         <v>0</v>
@@ -1223,7 +1232,7 @@
         <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1232,20 +1241,22 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>37</v>
+        <v>181</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>39</v>
+        <v>180</v>
       </c>
       <c r="D7" s="6">
         <v>0</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" t="s">
-        <v>174</v>
+      <c r="E7" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>182</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -1263,11 +1274,11 @@
         <v>39</v>
       </c>
       <c r="D8" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -1285,11 +1296,11 @@
         <v>39</v>
       </c>
       <c r="D9" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
@@ -1307,11 +1318,11 @@
         <v>39</v>
       </c>
       <c r="D10" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -1329,13 +1340,11 @@
         <v>39</v>
       </c>
       <c r="D11" s="6">
-        <v>4</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>179</v>
+        <v>3</v>
+      </c>
+      <c r="E11" s="6"/>
+      <c r="F11" t="s">
+        <v>158</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
@@ -1344,22 +1353,22 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="D12" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -1377,13 +1386,13 @@
         <v>72</v>
       </c>
       <c r="D13" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
@@ -1391,36 +1400,36 @@
       <c r="J13" s="6"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
+      <c r="A14" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="6">
+        <v>1</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>159</v>
+      </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" s="6">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>92</v>
-      </c>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
@@ -1437,13 +1446,13 @@
         <v>61</v>
       </c>
       <c r="D16" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
@@ -1461,13 +1470,13 @@
         <v>61</v>
       </c>
       <c r="D17" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
@@ -1485,13 +1494,13 @@
         <v>61</v>
       </c>
       <c r="D18" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
@@ -1509,13 +1518,13 @@
         <v>61</v>
       </c>
       <c r="D19" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>157</v>
+        <v>64</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -1533,13 +1542,13 @@
         <v>61</v>
       </c>
       <c r="D20" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>65</v>
+        <v>155</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
@@ -1557,13 +1566,13 @@
         <v>61</v>
       </c>
       <c r="D21" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>176</v>
+        <v>65</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
@@ -1572,22 +1581,22 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="D22" s="6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F22" t="s">
-        <v>175</v>
+      <c r="F22" s="6" t="s">
+        <v>174</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
@@ -1595,36 +1604,36 @@
       <c r="J22" s="6"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
+      <c r="A23" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" t="s">
+        <v>173</v>
+      </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6"/>
       <c r="J23" s="6"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D24" s="6">
-        <v>0</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>171</v>
-      </c>
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
@@ -1641,13 +1650,13 @@
         <v>42</v>
       </c>
       <c r="D25" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>43</v>
+        <v>169</v>
       </c>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
@@ -1665,13 +1674,13 @@
         <v>42</v>
       </c>
       <c r="D26" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F26" t="s">
-        <v>167</v>
+        <v>147</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
@@ -1689,13 +1698,13 @@
         <v>42</v>
       </c>
       <c r="D27" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F27" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
@@ -1713,13 +1722,13 @@
         <v>42</v>
       </c>
       <c r="D28" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F28" t="s">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
@@ -1728,22 +1737,22 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>149</v>
+        <v>41</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>150</v>
+        <v>42</v>
       </c>
       <c r="D29" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>173</v>
+        <v>147</v>
+      </c>
+      <c r="F29" t="s">
+        <v>139</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
@@ -1752,22 +1761,22 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
-        <v>44</v>
+        <v>148</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>45</v>
+        <v>149</v>
       </c>
       <c r="D30" s="6">
         <v>0</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>46</v>
+        <v>171</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="6"/>
@@ -1785,13 +1794,13 @@
         <v>45</v>
       </c>
       <c r="D31" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="6"/>
@@ -1809,13 +1818,13 @@
         <v>45</v>
       </c>
       <c r="D32" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
@@ -1824,22 +1833,22 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D33" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
@@ -1857,13 +1866,13 @@
         <v>50</v>
       </c>
       <c r="D34" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>147</v>
+        <v>51</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
@@ -1881,13 +1890,13 @@
         <v>50</v>
       </c>
       <c r="D35" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>52</v>
+        <v>146</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
@@ -1905,13 +1914,13 @@
         <v>50</v>
       </c>
       <c r="D36" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>146</v>
+        <v>52</v>
       </c>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
@@ -1929,13 +1938,13 @@
         <v>50</v>
       </c>
       <c r="D37" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>53</v>
+        <v>145</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
@@ -1944,22 +1953,22 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
-        <v>141</v>
+        <v>49</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>142</v>
+        <v>50</v>
       </c>
       <c r="D38" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F38" t="s">
-        <v>143</v>
+        <v>147</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>53</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
@@ -1968,75 +1977,75 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="6" t="s">
+      <c r="D39" s="6">
+        <v>0</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F39" t="s">
         <v>142</v>
       </c>
-      <c r="D39" s="6">
-        <v>1</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F39" t="s">
-        <v>144</v>
-      </c>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="6"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>142</v>
-      </c>
       <c r="D40" s="6">
+        <v>1</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F40" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D41" s="6">
         <v>2</v>
       </c>
-      <c r="E40" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F40" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="6"/>
-      <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
+      <c r="E41" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F41" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D42" s="6">
-        <v>0</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F42" t="s">
-        <v>106</v>
-      </c>
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
       <c r="I42" s="6"/>
@@ -2053,13 +2062,13 @@
         <v>97</v>
       </c>
       <c r="D43" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F43" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
@@ -2077,13 +2086,13 @@
         <v>97</v>
       </c>
       <c r="D44" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
@@ -2101,13 +2110,13 @@
         <v>97</v>
       </c>
       <c r="D45" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F45" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
@@ -2125,13 +2134,13 @@
         <v>97</v>
       </c>
       <c r="D46" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F46" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
@@ -2140,22 +2149,22 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
-        <v>151</v>
+        <v>94</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>152</v>
+        <v>97</v>
       </c>
       <c r="D47" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F47" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
@@ -2164,13 +2173,13 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>98</v>
+        <v>151</v>
       </c>
       <c r="D48" s="6">
         <v>0</v>
@@ -2179,7 +2188,7 @@
         <v>100</v>
       </c>
       <c r="F48" t="s">
-        <v>101</v>
+        <v>152</v>
       </c>
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
@@ -2197,13 +2206,13 @@
         <v>98</v>
       </c>
       <c r="D49" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F49" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
@@ -2221,13 +2230,13 @@
         <v>98</v>
       </c>
       <c r="D50" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F50" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
@@ -2236,22 +2245,22 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D51" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F51" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
@@ -2269,13 +2278,13 @@
         <v>99</v>
       </c>
       <c r="D52" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F52" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
@@ -2293,13 +2302,13 @@
         <v>99</v>
       </c>
       <c r="D53" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F53" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -2317,13 +2326,13 @@
         <v>99</v>
       </c>
       <c r="D54" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F54" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
@@ -2332,22 +2341,22 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D55" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F55" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>
@@ -2365,14 +2374,18 @@
         <v>104</v>
       </c>
       <c r="D56" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F56" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
@@ -2385,38 +2398,34 @@
         <v>104</v>
       </c>
       <c r="D57" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F57" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A58" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D58" s="6">
+        <v>2</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F58" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A59" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="D59" s="6">
-        <v>0</v>
-      </c>
-      <c r="E59" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="F59" t="s">
-        <v>119</v>
-      </c>
-      <c r="G59" s="6"/>
-      <c r="H59" s="6"/>
-      <c r="I59" s="6"/>
-      <c r="J59" s="6"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
@@ -2426,16 +2435,16 @@
         <v>6</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D60" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F60" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
@@ -2450,16 +2459,16 @@
         <v>6</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D61" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F61" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
@@ -2474,16 +2483,16 @@
         <v>6</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D62" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F62" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
@@ -2498,16 +2507,16 @@
         <v>6</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D63" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F63" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
@@ -2516,22 +2525,22 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
-        <v>154</v>
+        <v>105</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="D64" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F64" t="s">
-        <v>156</v>
+        <v>124</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
@@ -2540,13 +2549,13 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B65" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="D65" s="6">
         <v>0</v>
@@ -2555,7 +2564,7 @@
         <v>120</v>
       </c>
       <c r="F65" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="G65" s="6"/>
       <c r="H65" s="6"/>
@@ -2564,22 +2573,22 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D66" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F66" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G66" s="6"/>
       <c r="H66" s="6"/>
@@ -2588,22 +2597,22 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D67" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F67" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G67" s="6"/>
       <c r="H67" s="6"/>
@@ -2612,22 +2621,22 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D68" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F68" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G68" s="6"/>
       <c r="H68" s="6"/>
@@ -2636,22 +2645,22 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D69" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F69" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G69" s="6"/>
       <c r="H69" s="6"/>
@@ -2660,22 +2669,22 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B70" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D70" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F70" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G70" s="6"/>
       <c r="H70" s="6"/>
@@ -2684,22 +2693,22 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B71" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D71" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F71" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="G71" s="6"/>
       <c r="H71" s="6"/>
@@ -2708,54 +2717,54 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D72" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>120</v>
       </c>
       <c r="F72" t="s">
-        <v>126</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="G72" s="6"/>
+      <c r="H72" s="6"/>
+      <c r="I72" s="6"/>
+      <c r="J72" s="6"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A73" s="6"/>
-      <c r="B73" s="6"/>
-      <c r="C73" s="6"/>
-      <c r="D73" s="6"/>
-      <c r="E73" s="6"/>
+      <c r="A73" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D73" s="6">
+        <v>1</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F73" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A74" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B74" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D74" s="6">
-        <v>0</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="G74" s="6"/>
-      <c r="H74" s="6"/>
-      <c r="I74" s="6"/>
-      <c r="J74" s="6"/>
+      <c r="A74" s="6"/>
+      <c r="B74" s="6"/>
+      <c r="C74" s="6"/>
+      <c r="D74" s="6"/>
+      <c r="E74" s="6"/>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
@@ -2768,13 +2777,13 @@
         <v>67</v>
       </c>
       <c r="D75" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
@@ -2792,13 +2801,13 @@
         <v>67</v>
       </c>
       <c r="D76" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
@@ -2807,22 +2816,22 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D77" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="G77" s="6"/>
       <c r="H77" s="6"/>
@@ -2830,36 +2839,36 @@
       <c r="J77" s="6"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A78" s="6"/>
-      <c r="B78" s="6"/>
-      <c r="C78" s="6"/>
-      <c r="D78" s="6"/>
-      <c r="E78" s="6"/>
-      <c r="F78" s="6"/>
+      <c r="A78" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D78" s="6">
+        <v>0</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>70</v>
+      </c>
       <c r="G78" s="6"/>
       <c r="H78" s="6"/>
       <c r="I78" s="6"/>
       <c r="J78" s="6"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A79" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B79" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D79" s="6">
-        <v>0</v>
-      </c>
-      <c r="E79" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F79" s="6" t="s">
-        <v>75</v>
-      </c>
+      <c r="A79" s="6"/>
+      <c r="B79" s="6"/>
+      <c r="C79" s="6"/>
+      <c r="D79" s="6"/>
+      <c r="E79" s="6"/>
+      <c r="F79" s="6"/>
       <c r="G79" s="6"/>
       <c r="H79" s="6"/>
       <c r="I79" s="6"/>
@@ -2867,13 +2876,13 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D80" s="6">
         <v>0</v>
@@ -2882,7 +2891,7 @@
         <v>40</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>177</v>
+        <v>75</v>
       </c>
       <c r="G80" s="6"/>
       <c r="H80" s="6"/>
@@ -2891,22 +2900,22 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D81" s="6">
         <v>0</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="G81" s="6"/>
       <c r="H81" s="6"/>
@@ -2915,22 +2924,22 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D82" s="6">
         <v>0</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>84</v>
+        <v>160</v>
       </c>
       <c r="G82" s="6"/>
       <c r="H82" s="6"/>
@@ -2938,36 +2947,40 @@
       <c r="J82" s="6"/>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A83" s="6"/>
-      <c r="B83" s="6"/>
-      <c r="C83" s="6"/>
-      <c r="D83" s="6"/>
-      <c r="E83" s="6"/>
-      <c r="F83" s="6"/>
+      <c r="A83" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D83" s="6">
+        <v>0</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>84</v>
+      </c>
       <c r="G83" s="6"/>
       <c r="H83" s="6"/>
       <c r="I83" s="6"/>
       <c r="J83" s="6"/>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>85</v>
-      </c>
-      <c r="B84" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C84" t="s">
-        <v>86</v>
-      </c>
-      <c r="D84">
-        <v>0</v>
-      </c>
-      <c r="E84" t="s">
-        <v>40</v>
-      </c>
-      <c r="F84" t="s">
-        <v>88</v>
-      </c>
+      <c r="A84" s="6"/>
+      <c r="B84" s="6"/>
+      <c r="C84" s="6"/>
+      <c r="D84" s="6"/>
+      <c r="E84" s="6"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="6"/>
+      <c r="H84" s="6"/>
+      <c r="I84" s="6"/>
+      <c r="J84" s="6"/>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
@@ -2980,13 +2993,13 @@
         <v>86</v>
       </c>
       <c r="D85">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E85" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="F85" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
@@ -3000,13 +3013,13 @@
         <v>86</v>
       </c>
       <c r="D86">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E86" t="s">
         <v>87</v>
       </c>
       <c r="F86" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
@@ -3020,21 +3033,34 @@
         <v>86</v>
       </c>
       <c r="D87">
+        <v>2</v>
+      </c>
+      <c r="E87" t="s">
+        <v>87</v>
+      </c>
+      <c r="F87" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>85</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C88" t="s">
+        <v>86</v>
+      </c>
+      <c r="D88">
         <v>3</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E88" t="s">
         <v>40</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F88" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A93" s="6"/>
-      <c r="B93" s="6"/>
-      <c r="C93" s="6"/>
-      <c r="D93" s="6"/>
-      <c r="E93" s="6"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="6"/>
@@ -3043,6 +3069,13 @@
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
     </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A95" s="6"/>
+      <c r="B95" s="6"/>
+      <c r="C95" s="6"/>
+      <c r="D95" s="6"/>
+      <c r="E95" s="6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: Clean up not used Dialogue for ghost
</commit_message>
<xml_diff>
--- a/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
+++ b/Assets/Dialogue/Import/AllDialogue Worksheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR\Unity Projects\Class Assignments\CS 425\CS425-Senior-Project\Assets\Dialogue\Import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C02381-D37A-4F00-B6A6-D3F5B44253B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32FC9BF3-7814-4004-B12B-2960F9018B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="1440" windowWidth="18432" windowHeight="12540" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -569,7 +569,7 @@
     <t>ghostBlockedBeforeGateClue.asset</t>
   </si>
   <si>
-    <t>I don't want to talk to them right now. I just want to get out of here.</t>
+    <t>I don't want to talk to the ghost right now. I just want to get out of here.</t>
   </si>
 </sst>
 </file>

</xml_diff>